<commit_message>
merging remote into local
</commit_message>
<xml_diff>
--- a/single_mabs/4PL_edge_effects/model_tracker.xlsx
+++ b/single_mabs/4PL_edge_effects/model_tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhaddock\repos\automated_run_models\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhaddock\repos\bnAb_pnlme\single_mabs\4PL_edge_effects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD6408C9-9E7A-4F2B-905F-D08D3417BAD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{131BFB83-8F33-45E5-849A-85E38B90CB67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="375" yWindow="345" windowWidth="19185" windowHeight="10200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1128" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1230" uniqueCount="84">
   <si>
     <t>m0</t>
   </si>
@@ -254,6 +254,24 @@
   </si>
   <si>
     <t>k</t>
+  </si>
+  <si>
+    <t>m65</t>
+  </si>
+  <si>
+    <t>m66</t>
+  </si>
+  <si>
+    <t>m67</t>
+  </si>
+  <si>
+    <t>m68</t>
+  </si>
+  <si>
+    <t>m69</t>
+  </si>
+  <si>
+    <t>m70</t>
   </si>
 </sst>
 </file>
@@ -632,13 +650,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BO18"/>
+  <dimension ref="A1:BU18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:73" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>0</v>
       </c>
@@ -834,13 +852,31 @@
       <c r="BO1" t="s">
         <v>64</v>
       </c>
+      <c r="BP1" t="s">
+        <v>78</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>79</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>80</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>81</v>
+      </c>
+      <c r="BT1" t="s">
+        <v>82</v>
+      </c>
+      <c r="BU1" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="2" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:67" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:73" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>66</v>
       </c>
@@ -1042,8 +1078,26 @@
       <c r="BO3" s="1" t="s">
         <v>68</v>
       </c>
+      <c r="BP3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR3" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BS3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT3" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BU3" s="1" t="s">
+        <v>68</v>
+      </c>
     </row>
-    <row r="4" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:73" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>70</v>
       </c>
@@ -1242,8 +1296,26 @@
       <c r="BO4" t="s">
         <v>68</v>
       </c>
+      <c r="BP4" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ4" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR4" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS4" t="s">
+        <v>68</v>
+      </c>
+      <c r="BT4" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU4" t="s">
+        <v>68</v>
+      </c>
     </row>
-    <row r="5" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:73" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>71</v>
       </c>
@@ -1442,8 +1514,26 @@
       <c r="BO5" t="s">
         <v>68</v>
       </c>
+      <c r="BP5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BQ5" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR5" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BT5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BU5" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="6" spans="1:67" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:73" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>72</v>
       </c>
@@ -1645,8 +1735,26 @@
       <c r="BO6" s="1" t="s">
         <v>69</v>
       </c>
+      <c r="BP6" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ6" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR6" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS6" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT6" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU6" s="1" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="7" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:73" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>70</v>
       </c>
@@ -1845,8 +1953,26 @@
       <c r="BO7" t="s">
         <v>69</v>
       </c>
+      <c r="BP7" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ7" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR7" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS7" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT7" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU7" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="8" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:73" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>71</v>
       </c>
@@ -2045,8 +2171,26 @@
       <c r="BO8" t="s">
         <v>69</v>
       </c>
+      <c r="BP8" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ8" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR8" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS8" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT8" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU8" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="9" spans="1:67" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:73" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>73</v>
       </c>
@@ -2248,8 +2392,26 @@
       <c r="BO9" s="1" t="s">
         <v>69</v>
       </c>
+      <c r="BP9" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ9" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR9" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS9" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT9" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU9" s="1" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="10" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:73" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>70</v>
       </c>
@@ -2448,8 +2610,26 @@
       <c r="BO10" t="s">
         <v>69</v>
       </c>
+      <c r="BP10" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ10" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR10" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS10" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT10" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU10" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="11" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:73" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>71</v>
       </c>
@@ -2648,8 +2828,26 @@
       <c r="BO11" t="s">
         <v>69</v>
       </c>
+      <c r="BP11" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ11" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR11" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS11" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT11" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU11" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="12" spans="1:67" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:73" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>74</v>
       </c>
@@ -2851,8 +3049,26 @@
       <c r="BO12" s="1" t="s">
         <v>69</v>
       </c>
+      <c r="BP12" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ12" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR12" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS12" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT12" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU12" s="1" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="13" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:73" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>70</v>
       </c>
@@ -3051,8 +3267,26 @@
       <c r="BO13" t="s">
         <v>68</v>
       </c>
+      <c r="BP13" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ13" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR13" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS13" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT13" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU13" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="14" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:73" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>71</v>
       </c>
@@ -3251,8 +3485,26 @@
       <c r="BO14" t="s">
         <v>69</v>
       </c>
+      <c r="BP14" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ14" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR14" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS14" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT14" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU14" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="15" spans="1:67" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:73" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>75</v>
       </c>
@@ -3454,8 +3706,26 @@
       <c r="BO15" s="1" t="s">
         <v>68</v>
       </c>
+      <c r="BP15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BQ15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BS15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BT15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BU15" s="1" t="s">
+        <v>68</v>
+      </c>
     </row>
-    <row r="16" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:73" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>76</v>
       </c>
@@ -3654,8 +3924,26 @@
       <c r="BO16" t="s">
         <v>69</v>
       </c>
+      <c r="BP16" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ16" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR16" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS16" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT16" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU16" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="17" spans="1:67" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:73" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>77</v>
       </c>
@@ -3857,8 +4145,26 @@
       <c r="BO17" s="1" t="s">
         <v>68</v>
       </c>
+      <c r="BP17" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BQ17" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR17" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BS17" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BT17" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BU17" s="1" t="s">
+        <v>68</v>
+      </c>
     </row>
-    <row r="18" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:73" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>76</v>
       </c>
@@ -4055,6 +4361,24 @@
         <v>69</v>
       </c>
       <c r="BO18" t="s">
+        <v>69</v>
+      </c>
+      <c r="BP18" t="s">
+        <v>69</v>
+      </c>
+      <c r="BQ18" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR18" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS18" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT18" t="s">
+        <v>69</v>
+      </c>
+      <c r="BU18" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>